<commit_message>
Initial commit on Navigator UI Changes branch
</commit_message>
<xml_diff>
--- a/AI_TOOLS_Roles.xlsx
+++ b/AI_TOOLS_Roles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Ashok.Pottapalli/Desktop/AI_ML/Navigator UI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3693DEF1-4E74-4C44-B386-7759A80C6854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9B337EC-400F-DC4F-B8D8-736536F94727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -878,9 +878,6 @@
     <t>General-purpose AI for writing, reasoning, summarization, and Q&amp;A.</t>
   </si>
   <si>
-    <t>/static/chatgpt.png</t>
-  </si>
-  <si>
     <t>Microsoft Copilot</t>
   </si>
   <si>
@@ -893,9 +890,6 @@
     <t>AI assistant integrated with Microsoft 365 for everyday work productivity.</t>
   </si>
   <si>
-    <t>/static/microsoft%20copilot.jpeg</t>
-  </si>
-  <si>
     <t>Cassidy</t>
   </si>
   <si>
@@ -908,9 +902,6 @@
     <t>Automates business workflows and system integrations using AI.</t>
   </si>
   <si>
-    <t>/static/cassidy.png</t>
-  </si>
-  <si>
     <t>Jasper</t>
   </si>
   <si>
@@ -923,9 +914,6 @@
     <t>Generates marketing content at scale with brand control.</t>
   </si>
   <si>
-    <t>/static/jasper.png</t>
-  </si>
-  <si>
     <t>Synthesia</t>
   </si>
   <si>
@@ -938,9 +926,6 @@
     <t>Creates training and explainer videos using AI avatars</t>
   </si>
   <si>
-    <t>/static/synthesia.svg</t>
-  </si>
-  <si>
     <t>Clay</t>
   </si>
   <si>
@@ -953,9 +938,6 @@
     <t>Enriches lead data and powers outbound sales workflows.</t>
   </si>
   <si>
-    <t>/static/Clay.png</t>
-  </si>
-  <si>
     <t>Icertis</t>
   </si>
   <si>
@@ -968,9 +950,6 @@
     <t>Manages contracts and identifies risk using AI.</t>
   </si>
   <si>
-    <t>/static/icertis-logo.svg</t>
-  </si>
-  <si>
     <t>HubSpot</t>
   </si>
   <si>
@@ -983,16 +962,37 @@
     <t>CRM platform with AI for marketing, sales, and customer service.</t>
   </si>
   <si>
-    <t>/static/hubspot.png</t>
-  </si>
-  <si>
-    <t>/static/Sherlock.png</t>
-  </si>
-  <si>
-    <t>/static/aXet.svg</t>
-  </si>
-  <si>
-    <t>/static/Navigator.svg</t>
+    <t>/static/Images/Navigator.svg</t>
+  </si>
+  <si>
+    <t>/static/Images/aXet.svg</t>
+  </si>
+  <si>
+    <t>/static/Images/Sherlock.png</t>
+  </si>
+  <si>
+    <t>/static/Images/chatgpt.png</t>
+  </si>
+  <si>
+    <t>/static/Images/microsoft%20copilot.jpeg</t>
+  </si>
+  <si>
+    <t>/static/Images/cassidy.png</t>
+  </si>
+  <si>
+    <t>/static/Images/jasper.png</t>
+  </si>
+  <si>
+    <t>/static/Images/synthesia.svg</t>
+  </si>
+  <si>
+    <t>/static/Images/Clay.png</t>
+  </si>
+  <si>
+    <t>/static/Images/icertis-logo.svg</t>
+  </si>
+  <si>
+    <t>/static/Images/hubspot.png</t>
   </si>
 </sst>
 </file>
@@ -1509,7 +1509,7 @@
         <v>46</v>
       </c>
       <c r="Y2" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.2">
@@ -1580,7 +1580,7 @@
         <v>62</v>
       </c>
       <c r="Y3" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.2">
@@ -1654,7 +1654,7 @@
         <v>81</v>
       </c>
       <c r="Y4" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.2">
@@ -1728,7 +1728,7 @@
         <v>97</v>
       </c>
       <c r="Y5" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.2">
@@ -1799,7 +1799,7 @@
         <v>112</v>
       </c>
       <c r="Y6" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.2">
@@ -1876,7 +1876,7 @@
         <v>128</v>
       </c>
       <c r="Y7" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.2">
@@ -1953,7 +1953,7 @@
         <v>143</v>
       </c>
       <c r="Y8" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.2">
@@ -2024,7 +2024,7 @@
         <v>158</v>
       </c>
       <c r="Y9" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.2">
@@ -2095,7 +2095,7 @@
         <v>173</v>
       </c>
       <c r="Y10" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.2">
@@ -2166,7 +2166,7 @@
         <v>190</v>
       </c>
       <c r="Y11" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.2">
@@ -2240,7 +2240,7 @@
         <v>208</v>
       </c>
       <c r="Y12" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.2">
@@ -2311,7 +2311,7 @@
         <v>225</v>
       </c>
       <c r="Y13" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.2">
@@ -2385,7 +2385,7 @@
         <v>244</v>
       </c>
       <c r="Y14" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.2">
@@ -2456,7 +2456,7 @@
         <v>260</v>
       </c>
       <c r="Y15" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.2">
@@ -2473,126 +2473,126 @@
         <v>264</v>
       </c>
       <c r="Y16" t="s">
-        <v>265</v>
+        <v>296</v>
       </c>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>265</v>
+      </c>
+      <c r="B17" t="s">
         <v>266</v>
       </c>
-      <c r="B17" t="s">
+      <c r="S17" t="s">
         <v>267</v>
       </c>
-      <c r="S17" t="s">
+      <c r="X17" t="s">
         <v>268</v>
       </c>
-      <c r="X17" t="s">
-        <v>269</v>
-      </c>
       <c r="Y17" t="s">
-        <v>270</v>
+        <v>297</v>
       </c>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>269</v>
+      </c>
+      <c r="B18" t="s">
+        <v>270</v>
+      </c>
+      <c r="S18" t="s">
         <v>271</v>
       </c>
-      <c r="B18" t="s">
+      <c r="X18" t="s">
         <v>272</v>
       </c>
-      <c r="S18" t="s">
-        <v>273</v>
-      </c>
-      <c r="X18" t="s">
-        <v>274</v>
-      </c>
       <c r="Y18" t="s">
-        <v>275</v>
+        <v>298</v>
       </c>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>273</v>
+      </c>
+      <c r="B19" t="s">
+        <v>274</v>
+      </c>
+      <c r="S19" t="s">
+        <v>275</v>
+      </c>
+      <c r="X19" t="s">
         <v>276</v>
       </c>
-      <c r="B19" t="s">
-        <v>277</v>
-      </c>
-      <c r="S19" t="s">
-        <v>278</v>
-      </c>
-      <c r="X19" t="s">
-        <v>279</v>
-      </c>
       <c r="Y19" t="s">
-        <v>280</v>
+        <v>299</v>
       </c>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="B20" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="S20" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="X20" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="Y20" t="s">
-        <v>285</v>
+        <v>300</v>
       </c>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="B21" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="S21" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="X21" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="Y21" t="s">
-        <v>290</v>
+        <v>301</v>
       </c>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="B22" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="S22" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="X22" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="Y22" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="B23" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="S23" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="X23" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="Y23" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
   </sheetData>

</xml_diff>